<commit_message>
Update WGINOR xlsx data file (typos)
</commit_message>
<xml_diff>
--- a/TAF_ATAC/boot/data/WGINOR_Dataset_2025.xlsx
+++ b/TAF_ATAC/boot/data/WGINOR_Dataset_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjamin/Documents/Work/divers/Conferences_and_workshops/ICES_expert_groups/WGINOR/WGINOR_Git/WGINOR/TAF_ATAC/boot/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjamin/Documents/Work/divers/Conferences_and_workshops/ICES_expert_groups/WGINOR/WGINOR_Git/WGINOR/TAF_ATAC/boot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB95D982-C44F-3149-9C04-698E3704E3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE789E8F-F867-9F4C-A80C-1EEB594139DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="38640" windowHeight="26140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MetaMetaData" sheetId="10" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2535" uniqueCount="1110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2535" uniqueCount="1109">
   <si>
     <t>MetaDataKey</t>
   </si>
@@ -3553,9 +3553,6 @@
   </si>
   <si>
     <t>Year</t>
-  </si>
-  <si>
-    <t>RelativeHearContent</t>
   </si>
   <si>
     <t>NA</t>
@@ -15096,7 +15093,7 @@
         <v>290</v>
       </c>
       <c r="R1" s="50" t="s">
-        <v>1105</v>
+        <v>309</v>
       </c>
       <c r="S1" s="50" t="s">
         <v>321</v>
@@ -26009,7 +26006,7 @@
         <v>8222</v>
       </c>
       <c r="AE96" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="AK96" s="79">
         <v>15291</v>
@@ -32768,7 +32765,7 @@
         <v>2024</v>
       </c>
       <c r="B119" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="C119" s="1">
         <v>0.54100000000000004</v>
@@ -32945,10 +32942,10 @@
         <v>415</v>
       </c>
       <c r="BX119" t="s">
+        <v>1107</v>
+      </c>
+      <c r="BY119" t="s">
         <v>1108</v>
-      </c>
-      <c r="BY119" t="s">
-        <v>1109</v>
       </c>
       <c r="BZ119" s="55">
         <v>7.87</v>
@@ -33167,14 +33164,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="23f0569d-6e96-4da0-8a6f-de089bfd7312" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e325a71-b6a2-4928-b4aa-411584cbd42f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -33413,7 +33403,14 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="23f0569d-6e96-4da0-8a6f-de089bfd7312" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e325a71-b6a2-4928-b4aa-411584cbd42f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -33426,18 +33423,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50E9B672-0F7D-497D-93F7-112DAC958315}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0580923F-C6D6-4548-B6D5-050228A72A87}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="23f0569d-6e96-4da0-8a6f-de089bfd7312"/>
-    <ds:schemaRef ds:uri="1e325a71-b6a2-4928-b4aa-411584cbd42f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -33462,9 +33450,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0580923F-C6D6-4548-B6D5-050228A72A87}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50E9B672-0F7D-497D-93F7-112DAC958315}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="23f0569d-6e96-4da0-8a6f-de089bfd7312"/>
+    <ds:schemaRef ds:uri="1e325a71-b6a2-4928-b4aa-411584cbd42f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update time-series (units for catch values and fishing power) and run new fits
</commit_message>
<xml_diff>
--- a/TAF_ATAC/boot/data/WGINOR_Dataset_2025.xlsx
+++ b/TAF_ATAC/boot/data/WGINOR_Dataset_2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjamin/Documents/Work/divers/Conferences_and_workshops/ICES_expert_groups/WGINOR/WGINOR_Git/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benjamin/Documents/Work/divers/Conferences_and_workshops/ICES_expert_groups/WGINOR/WGINOR_Git/WGINOR/TAF_ATAC/boot/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4991AA-73E7-DC4B-B0ED-4785455837E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C92B94-7C3C-494E-B750-B5946720F05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="22420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="1106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2476" uniqueCount="1107">
   <si>
     <t>MetaDataKey</t>
   </si>
@@ -3384,21 +3384,6 @@
     <t>Release CO2 from shipping</t>
   </si>
   <si>
-    <r>
-      <t>tonne CO</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>2</t>
-    </r>
-  </si>
-  <si>
     <t>LicenseSalmonTrout</t>
   </si>
   <si>
@@ -3439,9 +3424,6 @@
   </si>
   <si>
     <t>Engine power</t>
-  </si>
-  <si>
-    <t>horse power</t>
   </si>
   <si>
     <t>NbFishermen</t>
@@ -3556,6 +3538,27 @@
   </si>
   <si>
     <t>ArcticWater</t>
+  </si>
+  <si>
+    <t>million NOK</t>
+  </si>
+  <si>
+    <r>
+      <t>thousand tonne CO</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+  </si>
+  <si>
+    <t>thousand horse power</t>
   </si>
 </sst>
 </file>
@@ -6336,7 +6339,7 @@
     </row>
     <row r="18" spans="1:39" ht="30" x14ac:dyDescent="0.2">
       <c r="A18" s="92" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>283</v>
@@ -6454,7 +6457,7 @@
     </row>
     <row r="20" spans="1:39" ht="328" x14ac:dyDescent="0.2">
       <c r="A20" s="92" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>286</v>
@@ -13557,7 +13560,7 @@
         <v>992</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F90" s="91" t="s">
         <v>189</v>
@@ -13628,7 +13631,7 @@
         <v>992</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F91" s="91" t="s">
         <v>189</v>
@@ -13699,7 +13702,7 @@
         <v>992</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F92" s="91" t="s">
         <v>189</v>
@@ -13770,7 +13773,7 @@
         <v>992</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F93" s="91" t="s">
         <v>189</v>
@@ -13841,7 +13844,7 @@
         <v>992</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F94" s="91" t="s">
         <v>189</v>
@@ -13912,7 +13915,7 @@
         <v>992</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F95" s="91" t="s">
         <v>189</v>
@@ -13983,7 +13986,7 @@
         <v>992</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>1039</v>
+        <v>1104</v>
       </c>
       <c r="F96" s="91" t="s">
         <v>189</v>
@@ -14171,7 +14174,7 @@
       <c r="AZ98" s="94"/>
       <c r="BA98" s="94"/>
     </row>
-    <row r="99" spans="1:53" ht="17" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:53" ht="32" x14ac:dyDescent="0.2">
       <c r="A99" s="112" t="s">
         <v>1054</v>
       </c>
@@ -14182,7 +14185,7 @@
         <v>992</v>
       </c>
       <c r="D99" s="107" t="s">
-        <v>1056</v>
+        <v>1105</v>
       </c>
       <c r="F99" s="91" t="s">
         <v>110</v>
@@ -14244,10 +14247,10 @@
     </row>
     <row r="100" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A100" s="111" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B100" s="3" t="s">
         <v>1057</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>1058</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>992</v>
@@ -14315,10 +14318,10 @@
     </row>
     <row r="101" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" s="111" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B101" s="3" t="s">
         <v>1059</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>1060</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>992</v>
@@ -14386,10 +14389,10 @@
     </row>
     <row r="102" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A102" s="111" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B102" s="3" t="s">
         <v>1061</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>1062</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>992</v>
@@ -14419,10 +14422,10 @@
     </row>
     <row r="103" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A103" s="111" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>1063</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>1064</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>992</v>
@@ -14452,10 +14455,10 @@
     </row>
     <row r="104" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" s="111" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B104" s="3" t="s">
         <v>1065</v>
-      </c>
-      <c r="B104" s="3" t="s">
-        <v>1066</v>
       </c>
       <c r="C104" s="3" t="s">
         <v>992</v>
@@ -14485,10 +14488,10 @@
     </row>
     <row r="105" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A105" s="111" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B105" s="3" t="s">
         <v>1067</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>1068</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>992</v>
@@ -14516,18 +14519,18 @@
         <v>992</v>
       </c>
     </row>
-    <row r="106" spans="1:53" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:53" ht="30" x14ac:dyDescent="0.2">
       <c r="A106" s="111" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B106" s="3" t="s">
         <v>1069</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>1070</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>992</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>1071</v>
+        <v>1106</v>
       </c>
       <c r="F106" s="91" t="s">
         <v>110</v>
@@ -14551,10 +14554,10 @@
     </row>
     <row r="107" spans="1:53" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="111" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>992</v>
@@ -14584,16 +14587,16 @@
     </row>
     <row r="108" spans="1:53" ht="17" x14ac:dyDescent="0.2">
       <c r="A108" s="111" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>661</v>
       </c>
       <c r="D108" s="107" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="F108" s="91" t="s">
         <v>189</v>
@@ -14609,71 +14612,71 @@
       </c>
       <c r="J108" s="4"/>
       <c r="O108" s="114" t="s">
+        <v>1075</v>
+      </c>
+      <c r="P108" s="114" t="s">
+        <v>1076</v>
+      </c>
+      <c r="Q108" s="114" t="s">
         <v>1077</v>
       </c>
-      <c r="P108" s="114" t="s">
+      <c r="R108" s="114" t="s">
         <v>1078</v>
       </c>
-      <c r="Q108" s="114" t="s">
+      <c r="S108" s="114" t="s">
         <v>1079</v>
       </c>
-      <c r="R108" s="114" t="s">
+      <c r="T108" s="114" t="s">
         <v>1080</v>
       </c>
-      <c r="S108" s="114" t="s">
+      <c r="U108" s="114" t="s">
         <v>1081</v>
       </c>
-      <c r="T108" s="114" t="s">
+      <c r="V108" s="114" t="s">
         <v>1082</v>
       </c>
-      <c r="U108" s="114" t="s">
+      <c r="W108" s="114" t="s">
         <v>1083</v>
       </c>
-      <c r="V108" s="114" t="s">
+      <c r="X108" s="114" t="s">
         <v>1084</v>
       </c>
-      <c r="W108" s="114" t="s">
+      <c r="Y108" s="114" t="s">
         <v>1085</v>
       </c>
-      <c r="X108" s="114" t="s">
+      <c r="Z108" s="114" t="s">
         <v>1086</v>
       </c>
-      <c r="Y108" s="114" t="s">
+      <c r="AA108" s="114" t="s">
         <v>1087</v>
-      </c>
-      <c r="Z108" s="114" t="s">
-        <v>1088</v>
-      </c>
-      <c r="AA108" s="114" t="s">
-        <v>1089</v>
       </c>
       <c r="AB108" s="114"/>
       <c r="AC108" s="114" t="s">
+        <v>1088</v>
+      </c>
+      <c r="AD108" s="114" t="s">
+        <v>1089</v>
+      </c>
+      <c r="AE108" s="114" t="s">
         <v>1090</v>
       </c>
-      <c r="AD108" s="114" t="s">
+      <c r="AF108" s="114" t="s">
         <v>1091</v>
       </c>
-      <c r="AE108" s="114" t="s">
+      <c r="AG108" s="114" t="s">
         <v>1092</v>
       </c>
-      <c r="AF108" s="114" t="s">
+      <c r="AH108" s="114" t="s">
         <v>1093</v>
       </c>
-      <c r="AG108" s="114" t="s">
+      <c r="AI108" s="114" t="s">
         <v>1094</v>
       </c>
-      <c r="AH108" s="114" t="s">
+      <c r="AJ108" s="114" t="s">
         <v>1095</v>
       </c>
-      <c r="AI108" s="114" t="s">
+      <c r="AK108" s="114" t="s">
         <v>1096</v>
-      </c>
-      <c r="AJ108" s="114" t="s">
-        <v>1097</v>
-      </c>
-      <c r="AK108" s="114" t="s">
-        <v>1098</v>
       </c>
       <c r="AL108" s="3">
         <v>1</v>
@@ -14796,21 +14799,20 @@
     <col min="83" max="83" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="84" max="84" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="85" max="86" width="19.1640625" customWidth="1"/>
-    <col min="87" max="87" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="17" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="17.1640625" bestFit="1" customWidth="1"/>
-    <col min="94" max="96" width="17.1640625" customWidth="1"/>
+    <col min="87" max="87" width="14.33203125" customWidth="1"/>
+    <col min="88" max="88" width="17.6640625" customWidth="1"/>
+    <col min="89" max="89" width="17.33203125" customWidth="1"/>
+    <col min="90" max="90" width="17" customWidth="1"/>
+    <col min="91" max="91" width="15.33203125" customWidth="1"/>
+    <col min="92" max="92" width="13.6640625" customWidth="1"/>
+    <col min="93" max="96" width="17.1640625" customWidth="1"/>
     <col min="97" max="97" width="14.5" bestFit="1" customWidth="1"/>
     <col min="98" max="98" width="12.5" bestFit="1" customWidth="1"/>
     <col min="99" max="99" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="100" max="100" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="101" max="101" width="14.5" bestFit="1" customWidth="1"/>
     <col min="102" max="102" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="103" max="103" width="13.6640625" customWidth="1"/>
     <col min="104" max="104" width="10" bestFit="1" customWidth="1"/>
     <col min="105" max="105" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="106" max="106" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -14818,7 +14820,7 @@
   <sheetData>
     <row r="1" spans="1:105" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="B1" s="50" t="s">
         <v>105</v>
@@ -14860,13 +14862,13 @@
         <v>280</v>
       </c>
       <c r="O1" s="50" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="P1" s="50" t="s">
         <v>284</v>
       </c>
       <c r="Q1" s="50" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="R1" s="50" t="s">
         <v>304</v>
@@ -15106,31 +15108,31 @@
         <v>1054</v>
       </c>
       <c r="CS1" s="54" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="CT1" s="54" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="CU1" s="54" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="CV1" s="54" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="CW1" s="54" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="CX1" s="54" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="CY1" s="54" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="CZ1" s="54" t="s">
+        <v>1070</v>
+      </c>
+      <c r="DA1" s="54" t="s">
         <v>1072</v>
-      </c>
-      <c r="DA1" s="54" t="s">
-        <v>1074</v>
       </c>
     </row>
     <row r="2" spans="1:105" x14ac:dyDescent="0.2">
@@ -20702,7 +20704,7 @@
         <v>13801</v>
       </c>
       <c r="CY66">
-        <v>482838</v>
+        <v>483</v>
       </c>
     </row>
     <row r="67" spans="1:104" x14ac:dyDescent="0.2">
@@ -20815,7 +20817,7 @@
         <v>13895</v>
       </c>
       <c r="CY67">
-        <v>511328</v>
+        <v>511</v>
       </c>
     </row>
     <row r="68" spans="1:104" x14ac:dyDescent="0.2">
@@ -20932,7 +20934,7 @@
         <v>12138</v>
       </c>
       <c r="CY68">
-        <v>525432</v>
+        <v>525</v>
       </c>
     </row>
     <row r="69" spans="1:104" x14ac:dyDescent="0.2">
@@ -21049,7 +21051,7 @@
         <v>12684</v>
       </c>
       <c r="CY69">
-        <v>563886</v>
+        <v>564</v>
       </c>
     </row>
     <row r="70" spans="1:104" x14ac:dyDescent="0.2">
@@ -21166,7 +21168,7 @@
         <v>12943</v>
       </c>
       <c r="CY70">
-        <v>608853</v>
+        <v>609</v>
       </c>
     </row>
     <row r="71" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -21287,7 +21289,7 @@
         <v>12881</v>
       </c>
       <c r="CY71">
-        <v>626146</v>
+        <v>626</v>
       </c>
     </row>
     <row r="72" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -21408,7 +21410,7 @@
         <v>11127</v>
       </c>
       <c r="CY72">
-        <v>653449</v>
+        <v>653</v>
       </c>
     </row>
     <row r="73" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -21531,7 +21533,7 @@
         <v>11095</v>
       </c>
       <c r="CY73">
-        <v>708185</v>
+        <v>708</v>
       </c>
     </row>
     <row r="74" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -21654,7 +21656,7 @@
         <v>11344</v>
       </c>
       <c r="CY74">
-        <v>722762</v>
+        <v>723</v>
       </c>
     </row>
     <row r="75" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -21783,7 +21785,7 @@
         <v>11594</v>
       </c>
       <c r="CY75">
-        <v>717640</v>
+        <v>718</v>
       </c>
       <c r="CZ75">
         <v>34789</v>
@@ -21937,7 +21939,7 @@
         <v>11456</v>
       </c>
       <c r="CY76">
-        <v>702034</v>
+        <v>702</v>
       </c>
     </row>
     <row r="77" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22084,7 +22086,7 @@
         <v>11390</v>
       </c>
       <c r="CY77">
-        <v>723381</v>
+        <v>723</v>
       </c>
     </row>
     <row r="78" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22237,7 +22239,7 @@
         <v>10981</v>
       </c>
       <c r="CY78">
-        <v>726349</v>
+        <v>726</v>
       </c>
     </row>
     <row r="79" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22390,7 +22392,7 @@
         <v>10903</v>
       </c>
       <c r="CY79">
-        <v>744274</v>
+        <v>744</v>
       </c>
     </row>
     <row r="80" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22543,7 +22545,7 @@
         <v>10458</v>
       </c>
       <c r="CY80">
-        <v>748388</v>
+        <v>748</v>
       </c>
     </row>
     <row r="81" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22698,7 +22700,7 @@
         <v>10225</v>
       </c>
       <c r="CY81">
-        <v>769759</v>
+        <v>770</v>
       </c>
     </row>
     <row r="82" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -22853,7 +22855,7 @@
         <v>9853</v>
       </c>
       <c r="CY82">
-        <v>800040</v>
+        <v>800</v>
       </c>
     </row>
     <row r="83" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -23024,7 +23026,7 @@
         <v>9223</v>
       </c>
       <c r="CY83">
-        <v>813255</v>
+        <v>813</v>
       </c>
     </row>
     <row r="84" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -23195,7 +23197,7 @@
         <v>8121</v>
       </c>
       <c r="CY84">
-        <v>793237</v>
+        <v>793</v>
       </c>
     </row>
     <row r="85" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -23366,7 +23368,7 @@
         <v>7589</v>
       </c>
       <c r="CY85">
-        <v>761026</v>
+        <v>761</v>
       </c>
       <c r="CZ85">
         <v>27518</v>
@@ -23540,7 +23542,7 @@
         <v>7457</v>
       </c>
       <c r="CY86">
-        <v>755112</v>
+        <v>755</v>
       </c>
     </row>
     <row r="87" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -23713,7 +23715,7 @@
         <v>7451</v>
       </c>
       <c r="CY87">
-        <v>752682</v>
+        <v>753</v>
       </c>
     </row>
     <row r="88" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -23886,7 +23888,7 @@
         <v>7169</v>
       </c>
       <c r="CY88">
-        <v>757561</v>
+        <v>758</v>
       </c>
     </row>
     <row r="89" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -24083,25 +24085,25 @@
       <c r="CG89" s="55"/>
       <c r="CH89" s="55"/>
       <c r="CI89">
-        <v>1132373</v>
+        <v>1132.373</v>
       </c>
       <c r="CJ89">
-        <v>965906</v>
+        <v>966</v>
       </c>
       <c r="CK89">
-        <v>212228</v>
+        <v>212</v>
       </c>
       <c r="CL89">
-        <v>4246143</v>
+        <v>4246</v>
       </c>
       <c r="CM89">
-        <v>657504</v>
+        <v>658</v>
       </c>
       <c r="CN89">
-        <v>958554</v>
+        <v>959</v>
       </c>
       <c r="CO89">
-        <v>189658</v>
+        <v>190</v>
       </c>
       <c r="CS89">
         <v>524</v>
@@ -24122,7 +24124,7 @@
         <v>6687</v>
       </c>
       <c r="CY89">
-        <v>758128</v>
+        <v>758</v>
       </c>
     </row>
     <row r="90" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -24334,25 +24336,25 @@
       <c r="CG90" s="55"/>
       <c r="CH90" s="55"/>
       <c r="CI90">
-        <v>1459189</v>
+        <v>1459.1890000000001</v>
       </c>
       <c r="CJ90">
-        <v>1034911</v>
+        <v>1035</v>
       </c>
       <c r="CK90">
-        <v>255845</v>
+        <v>256</v>
       </c>
       <c r="CL90">
-        <v>4173789</v>
+        <v>4174</v>
       </c>
       <c r="CM90">
-        <v>654912</v>
+        <v>655</v>
       </c>
       <c r="CN90">
-        <v>1328062</v>
+        <v>1328</v>
       </c>
       <c r="CO90">
-        <v>164661</v>
+        <v>165</v>
       </c>
       <c r="CS90">
         <v>519</v>
@@ -24373,7 +24375,7 @@
         <v>6328</v>
       </c>
       <c r="CY90">
-        <v>782754</v>
+        <v>783</v>
       </c>
     </row>
     <row r="91" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -24585,25 +24587,25 @@
       <c r="CG91" s="55"/>
       <c r="CH91" s="55"/>
       <c r="CI91">
-        <v>2154716</v>
+        <v>2154.7159999999999</v>
       </c>
       <c r="CJ91">
-        <v>1560031</v>
+        <v>1560</v>
       </c>
       <c r="CK91">
-        <v>320811</v>
+        <v>321</v>
       </c>
       <c r="CL91">
-        <v>3688694</v>
+        <v>3689</v>
       </c>
       <c r="CM91">
-        <v>723412</v>
+        <v>723</v>
       </c>
       <c r="CN91">
-        <v>1213183</v>
+        <v>1213</v>
       </c>
       <c r="CO91">
-        <v>222798</v>
+        <v>223</v>
       </c>
       <c r="CS91">
         <v>516</v>
@@ -24624,7 +24626,7 @@
         <v>6151</v>
       </c>
       <c r="CY91">
-        <v>784252</v>
+        <v>784</v>
       </c>
     </row>
     <row r="92" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -24836,25 +24838,25 @@
       <c r="CG92" s="55"/>
       <c r="CH92" s="55"/>
       <c r="CI92">
-        <v>2252233</v>
+        <v>2252.2330000000002</v>
       </c>
       <c r="CJ92">
-        <v>1592856</v>
+        <v>1593</v>
       </c>
       <c r="CK92">
-        <v>362097</v>
+        <v>362</v>
       </c>
       <c r="CL92">
-        <v>4094074</v>
+        <v>4094</v>
       </c>
       <c r="CM92">
-        <v>874791</v>
+        <v>875</v>
       </c>
       <c r="CN92">
-        <v>1014190</v>
+        <v>1014</v>
       </c>
       <c r="CO92">
-        <v>178011</v>
+        <v>178</v>
       </c>
       <c r="CS92">
         <v>509</v>
@@ -24875,7 +24877,7 @@
         <v>5943</v>
       </c>
       <c r="CY92">
-        <v>802641</v>
+        <v>803</v>
       </c>
     </row>
     <row r="93" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -25109,25 +25111,25 @@
       <c r="CG93" s="55"/>
       <c r="CH93" s="55"/>
       <c r="CI93">
-        <v>2045264</v>
+        <v>2045.2639999999999</v>
       </c>
       <c r="CJ93">
-        <v>1175927</v>
+        <v>1176</v>
       </c>
       <c r="CK93">
-        <v>684516</v>
+        <v>685</v>
       </c>
       <c r="CL93">
-        <v>4708982</v>
+        <v>4709</v>
       </c>
       <c r="CM93">
-        <v>1007890</v>
+        <v>1008</v>
       </c>
       <c r="CN93">
-        <v>1470938</v>
+        <v>1471</v>
       </c>
       <c r="CO93">
-        <v>275010</v>
+        <v>275</v>
       </c>
       <c r="CS93">
         <v>509</v>
@@ -25148,7 +25150,7 @@
         <v>5765</v>
       </c>
       <c r="CY93">
-        <v>811928</v>
+        <v>812</v>
       </c>
     </row>
     <row r="94" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -25382,25 +25384,25 @@
       <c r="CG94" s="55"/>
       <c r="CH94" s="55"/>
       <c r="CI94">
-        <v>1642760</v>
+        <v>1642.76</v>
       </c>
       <c r="CJ94">
-        <v>1182417</v>
+        <v>1182</v>
       </c>
       <c r="CK94">
-        <v>394631</v>
+        <v>395</v>
       </c>
       <c r="CL94">
-        <v>4542122</v>
+        <v>4542</v>
       </c>
       <c r="CM94">
-        <v>807484</v>
+        <v>807</v>
       </c>
       <c r="CN94">
-        <v>1383142</v>
+        <v>1383</v>
       </c>
       <c r="CO94">
-        <v>274680</v>
+        <v>275</v>
       </c>
       <c r="CS94">
         <v>512</v>
@@ -25421,7 +25423,7 @@
         <v>5751</v>
       </c>
       <c r="CY94">
-        <v>850914</v>
+        <v>851</v>
       </c>
     </row>
     <row r="95" spans="1:104" ht="16" x14ac:dyDescent="0.2">
@@ -25655,25 +25657,25 @@
       <c r="CG95" s="55"/>
       <c r="CH95" s="55"/>
       <c r="CI95">
-        <v>1902054</v>
+        <v>1902.0540000000001</v>
       </c>
       <c r="CJ95">
-        <v>1304551</v>
+        <v>1305</v>
       </c>
       <c r="CK95">
-        <v>428878</v>
+        <v>429</v>
       </c>
       <c r="CL95">
-        <v>3883428</v>
+        <v>3883</v>
       </c>
       <c r="CM95">
-        <v>706914</v>
+        <v>707</v>
       </c>
       <c r="CN95">
-        <v>979381</v>
+        <v>979</v>
       </c>
       <c r="CO95">
-        <v>232889</v>
+        <v>233</v>
       </c>
       <c r="CS95">
         <v>516</v>
@@ -25694,7 +25696,7 @@
         <v>5729</v>
       </c>
       <c r="CY95">
-        <v>871754</v>
+        <v>872</v>
       </c>
       <c r="CZ95">
         <v>20075</v>
@@ -25782,7 +25784,7 @@
         <v>8222</v>
       </c>
       <c r="AE96" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="AK96" s="79">
         <v>15291</v>
@@ -25931,25 +25933,25 @@
       <c r="CG96" s="55"/>
       <c r="CH96" s="55"/>
       <c r="CI96">
-        <v>2890332</v>
+        <v>2890.3319999999999</v>
       </c>
       <c r="CJ96">
-        <v>1722954</v>
+        <v>1723</v>
       </c>
       <c r="CK96">
-        <v>515946</v>
+        <v>516</v>
       </c>
       <c r="CL96">
-        <v>3739308</v>
+        <v>3739</v>
       </c>
       <c r="CM96">
-        <v>793516</v>
+        <v>794</v>
       </c>
       <c r="CN96">
-        <v>1058458</v>
+        <v>1058</v>
       </c>
       <c r="CO96">
-        <v>259977</v>
+        <v>260</v>
       </c>
       <c r="CS96">
         <v>511</v>
@@ -25970,7 +25972,7 @@
         <v>5403</v>
       </c>
       <c r="CY96">
-        <v>933379</v>
+        <v>933</v>
       </c>
     </row>
     <row r="97" spans="1:105" ht="16" x14ac:dyDescent="0.2">
@@ -26204,25 +26206,25 @@
       <c r="CG97" s="55"/>
       <c r="CH97" s="55"/>
       <c r="CI97">
-        <v>2591130</v>
+        <v>2591.13</v>
       </c>
       <c r="CJ97">
-        <v>1732431</v>
+        <v>1732</v>
       </c>
       <c r="CK97">
-        <v>700762</v>
+        <v>701</v>
       </c>
       <c r="CL97">
-        <v>3643620</v>
+        <v>3644</v>
       </c>
       <c r="CM97">
-        <v>702225</v>
+        <v>702</v>
       </c>
       <c r="CN97">
-        <v>1189422</v>
+        <v>1189</v>
       </c>
       <c r="CO97">
-        <v>139435</v>
+        <v>139</v>
       </c>
       <c r="CS97">
         <v>509</v>
@@ -26243,7 +26245,7 @@
         <v>4601</v>
       </c>
       <c r="CY97">
-        <v>923598</v>
+        <v>924</v>
       </c>
     </row>
     <row r="98" spans="1:105" ht="16" x14ac:dyDescent="0.2">
@@ -26485,25 +26487,25 @@
       <c r="CG98" s="55"/>
       <c r="CH98" s="55"/>
       <c r="CI98">
-        <v>1744721</v>
+        <v>1744.721</v>
       </c>
       <c r="CJ98">
-        <v>1248064</v>
+        <v>1248</v>
       </c>
       <c r="CK98">
-        <v>894157</v>
+        <v>894</v>
       </c>
       <c r="CL98">
-        <v>2897897</v>
+        <v>2898</v>
       </c>
       <c r="CM98">
-        <v>511623</v>
+        <v>512</v>
       </c>
       <c r="CN98">
-        <v>993743</v>
+        <v>994</v>
       </c>
       <c r="CO98">
-        <v>125534</v>
+        <v>126</v>
       </c>
       <c r="CS98">
         <v>521</v>
@@ -26524,7 +26526,7 @@
         <v>4328</v>
       </c>
       <c r="CY98">
-        <v>919021</v>
+        <v>919</v>
       </c>
       <c r="CZ98">
         <v>18645</v>
@@ -26769,25 +26771,25 @@
       <c r="CG99" s="55"/>
       <c r="CH99" s="55"/>
       <c r="CI99">
-        <v>2487953</v>
+        <v>2487.953</v>
       </c>
       <c r="CJ99">
-        <v>1640767</v>
+        <v>1641</v>
       </c>
       <c r="CK99">
-        <v>943078</v>
+        <v>943</v>
       </c>
       <c r="CL99">
-        <v>3437286</v>
+        <v>3437</v>
       </c>
       <c r="CM99">
-        <v>561815</v>
+        <v>562</v>
       </c>
       <c r="CN99">
-        <v>1034135</v>
+        <v>1034</v>
       </c>
       <c r="CO99">
-        <v>141990</v>
+        <v>142</v>
       </c>
       <c r="CS99">
         <v>545</v>
@@ -26808,7 +26810,7 @@
         <v>3591</v>
       </c>
       <c r="CY99">
-        <v>891790</v>
+        <v>892</v>
       </c>
       <c r="CZ99">
         <v>17334</v>
@@ -27053,25 +27055,25 @@
       <c r="CG100" s="55"/>
       <c r="CH100" s="55"/>
       <c r="CI100">
-        <v>3484007</v>
+        <v>3484.0070000000001</v>
       </c>
       <c r="CJ100">
-        <v>1816716</v>
+        <v>1817</v>
       </c>
       <c r="CK100">
-        <v>646170</v>
+        <v>646</v>
       </c>
       <c r="CL100">
-        <v>3626424</v>
+        <v>3626</v>
       </c>
       <c r="CM100">
-        <v>637843</v>
+        <v>638</v>
       </c>
       <c r="CN100">
-        <v>1338456</v>
+        <v>1338</v>
       </c>
       <c r="CO100">
-        <v>151454</v>
+        <v>151</v>
       </c>
       <c r="CS100">
         <v>541</v>
@@ -27092,7 +27094,7 @@
         <v>3386</v>
       </c>
       <c r="CY100">
-        <v>864419</v>
+        <v>864</v>
       </c>
       <c r="CZ100">
         <v>15519</v>
@@ -27337,25 +27339,25 @@
       <c r="CG101" s="55"/>
       <c r="CH101" s="55"/>
       <c r="CI101">
-        <v>2667319</v>
+        <v>2667.319</v>
       </c>
       <c r="CJ101">
-        <v>1159019</v>
+        <v>1159</v>
       </c>
       <c r="CK101">
-        <v>918353</v>
+        <v>918</v>
       </c>
       <c r="CL101">
-        <v>3925476</v>
+        <v>3925</v>
       </c>
       <c r="CM101">
-        <v>921093</v>
+        <v>921</v>
       </c>
       <c r="CN101">
-        <v>1656792</v>
+        <v>1657</v>
       </c>
       <c r="CO101">
-        <v>196215</v>
+        <v>196</v>
       </c>
       <c r="CS101">
         <v>547</v>
@@ -27376,7 +27378,7 @@
         <v>3201</v>
       </c>
       <c r="CY101">
-        <v>840613</v>
+        <v>841</v>
       </c>
       <c r="CZ101">
         <v>14708</v>
@@ -27624,25 +27626,25 @@
       <c r="CG102" s="55"/>
       <c r="CH102" s="55"/>
       <c r="CI102">
-        <v>2623639</v>
+        <v>2623.6390000000001</v>
       </c>
       <c r="CJ102">
-        <v>1155046</v>
+        <v>1155</v>
       </c>
       <c r="CK102">
-        <v>999979</v>
+        <v>1000</v>
       </c>
       <c r="CL102">
-        <v>4355224</v>
+        <v>4355</v>
       </c>
       <c r="CM102">
-        <v>991196</v>
+        <v>991</v>
       </c>
       <c r="CN102">
-        <v>1491584</v>
+        <v>1492</v>
       </c>
       <c r="CO102">
-        <v>118196</v>
+        <v>118</v>
       </c>
       <c r="CS102">
         <v>552</v>
@@ -27663,7 +27665,7 @@
         <v>3064</v>
       </c>
       <c r="CY102">
-        <v>808304</v>
+        <v>808</v>
       </c>
       <c r="CZ102">
         <v>14016</v>
@@ -27911,25 +27913,25 @@
       <c r="CG103" s="55"/>
       <c r="CH103" s="55"/>
       <c r="CI103">
-        <v>3188218</v>
+        <v>3188.2179999999998</v>
       </c>
       <c r="CJ103">
-        <v>1466209</v>
+        <v>1466</v>
       </c>
       <c r="CK103">
-        <v>481817</v>
+        <v>482</v>
       </c>
       <c r="CL103">
-        <v>4014892</v>
+        <v>4015</v>
       </c>
       <c r="CM103">
-        <v>735613</v>
+        <v>736</v>
       </c>
       <c r="CN103">
-        <v>1439249</v>
+        <v>1439</v>
       </c>
       <c r="CO103">
-        <v>75542</v>
+        <v>76</v>
       </c>
       <c r="CS103">
         <v>540</v>
@@ -27950,7 +27952,7 @@
         <v>2936</v>
       </c>
       <c r="CY103">
-        <v>810163</v>
+        <v>810</v>
       </c>
       <c r="CZ103">
         <v>13502</v>
@@ -28198,25 +28200,25 @@
       <c r="CG104" s="55"/>
       <c r="CH104" s="55"/>
       <c r="CI104">
-        <v>2987783</v>
+        <v>2987.7829999999999</v>
       </c>
       <c r="CJ104">
-        <v>1067997</v>
+        <v>1068</v>
       </c>
       <c r="CK104">
-        <v>351771</v>
+        <v>352</v>
       </c>
       <c r="CL104">
-        <v>3140464</v>
+        <v>3140</v>
       </c>
       <c r="CM104">
-        <v>921580</v>
+        <v>922</v>
       </c>
       <c r="CN104">
-        <v>1343288</v>
+        <v>1343</v>
       </c>
       <c r="CO104">
-        <v>68977</v>
+        <v>69</v>
       </c>
       <c r="CS104">
         <v>567</v>
@@ -28237,7 +28239,7 @@
         <v>2833</v>
       </c>
       <c r="CY104">
-        <v>812854</v>
+        <v>813</v>
       </c>
       <c r="CZ104">
         <v>13201</v>
@@ -28500,25 +28502,25 @@
       <c r="CG105" s="55"/>
       <c r="CH105" s="55"/>
       <c r="CI105">
-        <v>2981798</v>
+        <v>2981.7979999999998</v>
       </c>
       <c r="CJ105">
-        <v>1973149</v>
+        <v>1973</v>
       </c>
       <c r="CK105">
-        <v>394279</v>
+        <v>394</v>
       </c>
       <c r="CL105">
-        <v>3226104</v>
+        <v>3226</v>
       </c>
       <c r="CM105">
-        <v>1132536</v>
+        <v>1133</v>
       </c>
       <c r="CN105">
-        <v>1740866</v>
+        <v>1741</v>
       </c>
       <c r="CO105">
-        <v>134997</v>
+        <v>135</v>
       </c>
       <c r="CS105">
         <v>569</v>
@@ -28539,7 +28541,7 @@
         <v>2777</v>
       </c>
       <c r="CY105">
-        <v>798907</v>
+        <v>799</v>
       </c>
       <c r="CZ105">
         <v>12971</v>
@@ -28802,25 +28804,25 @@
       <c r="CG106" s="55"/>
       <c r="CH106" s="55"/>
       <c r="CI106">
-        <v>3572692</v>
+        <v>3572.692</v>
       </c>
       <c r="CJ106">
-        <v>2744390</v>
+        <v>2744</v>
       </c>
       <c r="CK106">
-        <v>70451</v>
+        <v>70</v>
       </c>
       <c r="CL106">
-        <v>4243752</v>
+        <v>4244</v>
       </c>
       <c r="CM106">
-        <v>1431521</v>
+        <v>1432</v>
       </c>
       <c r="CN106">
-        <v>1599878</v>
+        <v>1600</v>
       </c>
       <c r="CO106">
-        <v>119356</v>
+        <v>119</v>
       </c>
       <c r="CS106">
         <v>573</v>
@@ -28841,7 +28843,7 @@
         <v>2769</v>
       </c>
       <c r="CY106">
-        <v>824611</v>
+        <v>825</v>
       </c>
       <c r="CZ106">
         <v>12733</v>
@@ -29104,25 +29106,25 @@
       <c r="CG107" s="55"/>
       <c r="CH107" s="55"/>
       <c r="CI107">
-        <v>3792006</v>
+        <v>3792.0059999999999</v>
       </c>
       <c r="CJ107">
-        <v>1373920</v>
+        <v>1374</v>
       </c>
       <c r="CK107">
-        <v>294720</v>
+        <v>295</v>
       </c>
       <c r="CL107">
-        <v>4092453</v>
+        <v>4092</v>
       </c>
       <c r="CM107">
-        <v>1402112</v>
+        <v>1402</v>
       </c>
       <c r="CN107">
-        <v>1444463</v>
+        <v>1444</v>
       </c>
       <c r="CO107">
-        <v>110589</v>
+        <v>111</v>
       </c>
       <c r="CS107">
         <v>575</v>
@@ -29143,7 +29145,7 @@
         <v>2772</v>
       </c>
       <c r="CY107">
-        <v>808372</v>
+        <v>808</v>
       </c>
       <c r="CZ107">
         <v>12060</v>
@@ -29406,25 +29408,25 @@
       <c r="CG108" s="55"/>
       <c r="CH108" s="55"/>
       <c r="CI108">
-        <v>2535911</v>
+        <v>2535.9110000000001</v>
       </c>
       <c r="CJ108">
-        <v>1491617</v>
+        <v>1492</v>
       </c>
       <c r="CK108">
-        <v>401411</v>
+        <v>401</v>
       </c>
       <c r="CL108">
-        <v>4225350</v>
+        <v>4225</v>
       </c>
       <c r="CM108">
-        <v>1115570</v>
+        <v>1116</v>
       </c>
       <c r="CN108">
-        <v>989863</v>
+        <v>990</v>
       </c>
       <c r="CO108">
-        <v>81599</v>
+        <v>82</v>
       </c>
       <c r="CS108">
         <v>580</v>
@@ -29445,7 +29447,7 @@
         <v>2720</v>
       </c>
       <c r="CY108">
-        <v>816942</v>
+        <v>817</v>
       </c>
       <c r="CZ108">
         <v>11600</v>
@@ -29708,25 +29710,25 @@
       <c r="CG109" s="55"/>
       <c r="CH109" s="55"/>
       <c r="CI109">
-        <v>1962411</v>
+        <v>1962.4110000000001</v>
       </c>
       <c r="CJ109">
-        <v>1978353</v>
+        <v>1978</v>
       </c>
       <c r="CK109">
-        <v>591674</v>
+        <v>592</v>
       </c>
       <c r="CL109">
-        <v>4802784</v>
+        <v>4803</v>
       </c>
       <c r="CM109">
-        <v>1265488</v>
+        <v>1265</v>
       </c>
       <c r="CN109">
-        <v>1295925</v>
+        <v>1296</v>
       </c>
       <c r="CO109">
-        <v>193426</v>
+        <v>193</v>
       </c>
       <c r="CP109" s="15">
         <v>3.0643513789581203</v>
@@ -29753,7 +29755,7 @@
         <v>2663</v>
       </c>
       <c r="CY109">
-        <v>810643</v>
+        <v>811</v>
       </c>
       <c r="CZ109">
         <v>11282</v>
@@ -30016,25 +30018,25 @@
       <c r="CG110" s="55"/>
       <c r="CH110" s="55"/>
       <c r="CI110">
-        <v>1859690</v>
+        <v>1859.69</v>
       </c>
       <c r="CJ110">
-        <v>2029550</v>
+        <v>2030</v>
       </c>
       <c r="CK110">
-        <v>922868</v>
+        <v>923</v>
       </c>
       <c r="CL110">
-        <v>5722064</v>
+        <v>5722</v>
       </c>
       <c r="CM110">
-        <v>1141741</v>
+        <v>1142</v>
       </c>
       <c r="CN110">
-        <v>1489594</v>
+        <v>1490</v>
       </c>
       <c r="CO110">
-        <v>247955</v>
+        <v>248</v>
       </c>
       <c r="CP110" s="15">
         <v>678</v>
@@ -30061,7 +30063,7 @@
         <v>2591</v>
       </c>
       <c r="CY110">
-        <v>808012</v>
+        <v>808</v>
       </c>
       <c r="CZ110">
         <v>11129</v>
@@ -30324,25 +30326,25 @@
       <c r="CG111" s="55"/>
       <c r="CH111" s="55"/>
       <c r="CI111">
-        <v>2367289</v>
+        <v>2367.2890000000002</v>
       </c>
       <c r="CJ111">
-        <v>2348864</v>
+        <v>2349</v>
       </c>
       <c r="CK111">
-        <v>808715</v>
+        <v>809</v>
       </c>
       <c r="CL111">
-        <v>6225500</v>
+        <v>6226</v>
       </c>
       <c r="CM111">
-        <v>1135186</v>
+        <v>1135</v>
       </c>
       <c r="CN111">
-        <v>1378667</v>
+        <v>1379</v>
       </c>
       <c r="CO111">
-        <v>207852</v>
+        <v>208</v>
       </c>
       <c r="CP111" s="15">
         <v>2088.8030888030889</v>
@@ -30351,7 +30353,7 @@
         <v>3108.1081081081084</v>
       </c>
       <c r="CR111">
-        <v>1894793</v>
+        <v>1895</v>
       </c>
       <c r="CS111">
         <v>630</v>
@@ -30372,7 +30374,7 @@
         <v>2587</v>
       </c>
       <c r="CY111">
-        <v>794722</v>
+        <v>795</v>
       </c>
       <c r="CZ111">
         <v>11228</v>
@@ -30633,25 +30635,25 @@
       <c r="CG112" s="55"/>
       <c r="CH112" s="55"/>
       <c r="CI112">
-        <v>2177663</v>
+        <v>2177.663</v>
       </c>
       <c r="CJ112">
-        <v>1999593</v>
+        <v>2000</v>
       </c>
       <c r="CK112">
-        <v>549749</v>
+        <v>550</v>
       </c>
       <c r="CL112">
-        <v>6634092</v>
+        <v>6634</v>
       </c>
       <c r="CM112">
-        <v>1421438</v>
+        <v>1421</v>
       </c>
       <c r="CN112">
-        <v>1271068</v>
+        <v>1271</v>
       </c>
       <c r="CO112">
-        <v>211214</v>
+        <v>211</v>
       </c>
       <c r="CP112" s="15">
         <v>3653.0805687203792</v>
@@ -30660,7 +30662,7 @@
         <v>3575.355450236967</v>
       </c>
       <c r="CR112">
-        <v>1940823</v>
+        <v>1941</v>
       </c>
       <c r="CS112">
         <v>642</v>
@@ -30681,7 +30683,7 @@
         <v>2582</v>
       </c>
       <c r="CY112">
-        <v>798828</v>
+        <v>799</v>
       </c>
       <c r="CZ112">
         <v>11293</v>
@@ -30948,25 +30950,25 @@
         <v>4.6125461254612548</v>
       </c>
       <c r="CI113">
-        <v>1986788</v>
+        <v>1986.788</v>
       </c>
       <c r="CJ113">
-        <v>2284888</v>
+        <v>2285</v>
       </c>
       <c r="CK113">
-        <v>870835</v>
+        <v>871</v>
       </c>
       <c r="CL113">
-        <v>6706383</v>
+        <v>6706</v>
       </c>
       <c r="CM113">
-        <v>1406952</v>
+        <v>1407</v>
       </c>
       <c r="CN113">
-        <v>1346164</v>
+        <v>1346</v>
       </c>
       <c r="CO113">
-        <v>261589</v>
+        <v>262</v>
       </c>
       <c r="CP113" s="15">
         <v>1128.2287822878229</v>
@@ -30975,7 +30977,7 @@
         <v>6282.2878228782283</v>
       </c>
       <c r="CR113">
-        <v>2105001</v>
+        <v>2105</v>
       </c>
       <c r="CS113">
         <v>669</v>
@@ -30996,7 +30998,7 @@
         <v>2499</v>
       </c>
       <c r="CY113">
-        <v>808468</v>
+        <v>808</v>
       </c>
       <c r="CZ113">
         <v>11209</v>
@@ -31263,25 +31265,25 @@
         <v>4.512635379061372</v>
       </c>
       <c r="CI114">
-        <v>2323486</v>
+        <v>2323.4859999999999</v>
       </c>
       <c r="CJ114">
-        <v>2264071</v>
+        <v>2264</v>
       </c>
       <c r="CK114">
-        <v>796535</v>
+        <v>797</v>
       </c>
       <c r="CL114">
-        <v>6756282</v>
+        <v>6756</v>
       </c>
       <c r="CM114">
-        <v>1421548</v>
+        <v>1422</v>
       </c>
       <c r="CN114">
-        <v>1505347</v>
+        <v>1505</v>
       </c>
       <c r="CO114">
-        <v>294394</v>
+        <v>294</v>
       </c>
       <c r="CP114" s="15">
         <v>3836.6425992779787</v>
@@ -31290,7 +31292,7 @@
         <v>1588.447653429603</v>
       </c>
       <c r="CR114">
-        <v>2191532</v>
+        <v>2192</v>
       </c>
       <c r="CS114">
         <v>693</v>
@@ -31311,7 +31313,7 @@
         <v>2398</v>
       </c>
       <c r="CY114">
-        <v>822807</v>
+        <v>823</v>
       </c>
       <c r="CZ114">
         <v>11050</v>
@@ -31578,32 +31580,32 @@
         <v>0</v>
       </c>
       <c r="CI115">
-        <v>2803489</v>
+        <v>2803.489</v>
       </c>
       <c r="CJ115">
-        <v>2470222</v>
+        <v>2470</v>
       </c>
       <c r="CK115">
-        <v>1010442</v>
+        <v>1010</v>
       </c>
       <c r="CL115">
-        <v>6879328</v>
+        <v>6879</v>
       </c>
       <c r="CM115">
-        <v>1200623</v>
+        <v>1201</v>
       </c>
       <c r="CN115">
-        <v>1548832</v>
+        <v>1549</v>
       </c>
       <c r="CO115">
-        <v>314635</v>
+        <v>315</v>
       </c>
       <c r="CP115" s="15">
         <v>5802.139037433155</v>
       </c>
       <c r="CQ115" s="15"/>
       <c r="CR115">
-        <v>2006419</v>
+        <v>2006</v>
       </c>
       <c r="CS115">
         <v>725</v>
@@ -31624,7 +31626,7 @@
         <v>2339</v>
       </c>
       <c r="CY115">
-        <v>844634</v>
+        <v>845</v>
       </c>
       <c r="CZ115">
         <v>10973</v>
@@ -31883,25 +31885,25 @@
         <v>15.133505598621879</v>
       </c>
       <c r="CI116" s="15">
-        <v>3227983.6347975885</v>
+        <v>3227.9836347975884</v>
       </c>
       <c r="CJ116">
-        <v>2410492</v>
+        <v>2410</v>
       </c>
       <c r="CK116">
-        <v>511458</v>
+        <v>511</v>
       </c>
       <c r="CL116">
-        <v>6366506</v>
+        <v>6367</v>
       </c>
       <c r="CM116">
-        <v>1385372</v>
+        <v>1385</v>
       </c>
       <c r="CN116">
-        <v>1599903</v>
+        <v>1600</v>
       </c>
       <c r="CO116">
-        <v>307667</v>
+        <v>308</v>
       </c>
       <c r="CP116" s="15">
         <v>5937.1231696813093</v>
@@ -31910,7 +31912,7 @@
         <v>17496.124031007752</v>
       </c>
       <c r="CR116">
-        <v>2083058</v>
+        <v>2083</v>
       </c>
       <c r="CS116">
         <v>723</v>
@@ -31931,7 +31933,7 @@
         <v>2210</v>
       </c>
       <c r="CY116">
-        <v>858135</v>
+        <v>858</v>
       </c>
       <c r="CZ116">
         <v>10845</v>
@@ -32184,25 +32186,25 @@
         <v>15.789902280130294</v>
       </c>
       <c r="CI117" s="15">
-        <v>3258416.9381107492</v>
+        <v>3258.416938110749</v>
       </c>
       <c r="CJ117" s="15">
-        <v>3068453.5830618893</v>
+        <v>3068</v>
       </c>
       <c r="CK117" s="15">
-        <v>423437.29641693813</v>
+        <v>423</v>
       </c>
       <c r="CL117" s="15">
-        <v>8037285.8306188928</v>
+        <v>8037</v>
       </c>
       <c r="CM117" s="15">
-        <v>1382447.0684039088</v>
+        <v>1382</v>
       </c>
       <c r="CN117" s="15">
-        <v>2268983.713355049</v>
+        <v>2269</v>
       </c>
       <c r="CO117" s="15">
-        <v>469731.27035830618</v>
+        <v>470</v>
       </c>
       <c r="CP117" s="15">
         <v>6049.674267100977</v>
@@ -32211,7 +32213,7 @@
         <v>21092.019543973944</v>
       </c>
       <c r="CR117" s="15">
-        <v>2190775</v>
+        <v>2191</v>
       </c>
       <c r="CS117" s="15">
         <v>742</v>
@@ -32232,7 +32234,7 @@
         <v>2134</v>
       </c>
       <c r="CY117">
-        <v>849350</v>
+        <v>849</v>
       </c>
       <c r="CZ117">
         <v>10830</v>
@@ -32483,25 +32485,25 @@
         <v>13.734567901234568</v>
       </c>
       <c r="CI118" s="15">
-        <v>3647733.0246913582</v>
+        <v>3647.7330246913584</v>
       </c>
       <c r="CJ118" s="15">
-        <v>2925976.8518518498</v>
+        <v>2926</v>
       </c>
       <c r="CK118" s="15">
-        <v>995661.26543209876</v>
+        <v>996</v>
       </c>
       <c r="CL118" s="15">
-        <v>7294881.1728395065</v>
+        <v>7295</v>
       </c>
       <c r="CM118" s="15">
-        <v>1172679.0123456791</v>
+        <v>1173</v>
       </c>
       <c r="CN118" s="15">
-        <v>2346543.2098765434</v>
+        <v>2347</v>
       </c>
       <c r="CO118" s="15">
-        <v>545439.04320987652</v>
+        <v>545</v>
       </c>
       <c r="CP118" s="15">
         <v>6658.950617283951</v>
@@ -32510,7 +32512,7 @@
         <v>820.98765432098764</v>
       </c>
       <c r="CR118" s="15">
-        <v>2200216</v>
+        <v>2200</v>
       </c>
       <c r="CS118" s="15">
         <v>766</v>
@@ -32541,7 +32543,7 @@
         <v>2024</v>
       </c>
       <c r="B119" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="C119" s="1">
         <v>0.54100000000000004</v>
@@ -32718,10 +32720,10 @@
         <v>415</v>
       </c>
       <c r="BX119" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="BY119" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="BZ119" s="55">
         <v>7.87</v>
@@ -32751,25 +32753,25 @@
         <v>13.46</v>
       </c>
       <c r="CI119" s="15">
-        <v>3113440.8682634733</v>
+        <v>3113.4408682634735</v>
       </c>
       <c r="CJ119" s="15">
-        <v>4020647.4550898205</v>
+        <v>4021</v>
       </c>
       <c r="CK119" s="15">
-        <v>1014358.5329341318</v>
+        <v>1014</v>
       </c>
       <c r="CL119" s="15">
-        <v>5823776.1976047903</v>
+        <v>5824</v>
       </c>
       <c r="CM119" s="15">
-        <v>976605.53892215574</v>
+        <v>977</v>
       </c>
       <c r="CN119" s="15">
-        <v>1859436.3772455091</v>
+        <v>1859</v>
       </c>
       <c r="CO119" s="15">
-        <v>588941.61676646711</v>
+        <v>589</v>
       </c>
       <c r="CP119" s="15">
         <v>5921.4071856287428</v>
@@ -32778,7 +32780,7 @@
         <v>2616.0179640718566</v>
       </c>
       <c r="CR119" s="15">
-        <v>2263387</v>
+        <v>2263</v>
       </c>
       <c r="CS119" s="15">
         <v>777</v>
@@ -32936,21 +32938,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="23f0569d-6e96-4da0-8a6f-de089bfd7312" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e325a71-b6a2-4928-b4aa-411584cbd42f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010068F16C1DCC2C7F4BBF11888ACFCCDC13" ma:contentTypeVersion="15" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="1de7d766a3cc8f1c22612a8bf2a6bee0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e325a71-b6a2-4928-b4aa-411584cbd42f" xmlns:ns3="23f0569d-6e96-4da0-8a6f-de089bfd7312" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="26019dbb1fea1b515cb0ca62e7403dd3" ns2:_="" ns3:_="">
     <xsd:import namespace="1e325a71-b6a2-4928-b4aa-411584cbd42f"/>
@@ -33185,37 +33190,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="23f0569d-6e96-4da0-8a6f-de089bfd7312" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e325a71-b6a2-4928-b4aa-411584cbd42f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50E9B672-0F7D-497D-93F7-112DAC958315}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F42CBA7C-5EB8-43E9-9D2D-B8B85F9833C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="23f0569d-6e96-4da0-8a6f-de089bfd7312"/>
-    <ds:schemaRef ds:uri="1e325a71-b6a2-4928-b4aa-411584cbd42f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0580923F-C6D6-4548-B6D5-050228A72A87}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AFCC605C-31B5-4AA3-B84D-E35D5BDFAF8B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -33234,18 +33236,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0580923F-C6D6-4548-B6D5-050228A72A87}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50E9B672-0F7D-497D-93F7-112DAC958315}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F42CBA7C-5EB8-43E9-9D2D-B8B85F9833C3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="23f0569d-6e96-4da0-8a6f-de089bfd7312"/>
+    <ds:schemaRef ds:uri="1e325a71-b6a2-4928-b4aa-411584cbd42f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>